<commit_message>
XUSE: Add new parameters for ball mill process in CSV files
- Introduced two new variables: `Ball_Mill_Process_Param_Current_Cycle_Count` and `Ball_Mill_Process_Param_Current_Execution_Time` to both `xuse_variables.csv` and `xuse_variables_sim.csv`.
- These additions enhance the parameter set for monitoring and controlling the ball mill process, improving operational capabilities and data tracking.

These changes ensure that the XUSE device can now track the current cycle count and execution time for ball mill processes, facilitating better process management.
</commit_message>
<xml_diff>
--- a/unilabos/devices/workstation/XUSE/templates/球磨参数模板.xlsx
+++ b/unilabos/devices/workstation/XUSE/templates/球磨参数模板.xlsx
@@ -1,242 +1,177 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="8080"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="19200" windowHeight="8080" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="球磨" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="球磨" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
-  <si>
-    <t>参数名</t>
-  </si>
-  <si>
-    <t>参数值</t>
-  </si>
-  <si>
-    <t>步骤1_大盘转速</t>
-  </si>
-  <si>
-    <t>步骤1_工作时间</t>
-  </si>
-  <si>
-    <t>步骤2_大盘转速</t>
-  </si>
-  <si>
-    <t>步骤2_工作时间</t>
-  </si>
-  <si>
-    <t>步骤3_大盘转速</t>
-  </si>
-  <si>
-    <t>步骤3_工作时间</t>
-  </si>
-  <si>
-    <t>步骤4_大盘转速</t>
-  </si>
-  <si>
-    <t>步骤4_工作时间</t>
-  </si>
-  <si>
-    <t>步骤5_大盘转速</t>
-  </si>
-  <si>
-    <t>步骤5_工作时间</t>
-  </si>
-  <si>
-    <t>步骤6_大盘转速</t>
-  </si>
-  <si>
-    <t>步骤6_工作时间</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="20">
     <font>
-      <sz val="11"/>
+      <name val="宋体"/>
+      <charset val="134"/>
       <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
+      <b val="1"/>
+      <color theme="3"/>
       <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
       <color theme="3"/>
+      <sz val="15"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
+      <b val="1"/>
       <color theme="3"/>
+      <sz val="13"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
+      <b val="1"/>
       <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FF3F3F76"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color rgb="FF3F3F3F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FF9C0006"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FF9C6500"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color theme="0"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="33">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -537,153 +472,153 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -737,19 +672,75 @@
     <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
-</file>
-
-<file path=xl/customStorage/customStorage.xml><?xml version="1.0" encoding="utf-8"?>
-<customStorage xmlns="https://web.wps.cn/et/2018/main">
-  <book/>
-  <sheets/>
-</customStorage>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1035,84 +1026,121 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="15.1272727272727" customWidth="1"/>
+    <col width="15.1272727272727" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1">
-      <c r="A5" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1">
-      <c r="A6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1">
-      <c r="A7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1">
-      <c r="A8" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1">
-      <c r="A10" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1">
-      <c r="A11" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1">
-      <c r="A12" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1">
-      <c r="A13" t="s">
-        <v>13</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>参数名</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>参数值</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>步骤1_大盘转速</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>步骤1_工作时间</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>步骤2_大盘转速</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>步骤2_工作时间</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>步骤3_大盘转速</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>步骤3_工作时间</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>步骤4_大盘转速</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>步骤4_工作时间</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>步骤5_大盘转速</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>步骤5_工作时间</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>步骤6_大盘转速</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>步骤6_工作时间</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>当前工艺循环次数</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>